<commit_message>
Correct independent recommendations to EUR 29.675M without changing current prices
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -11869,7 +11869,7 @@
       </ns0:c>
       <ns0:c r="AF108" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG108" s="74" t="inlineStr">
@@ -11968,7 +11968,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC109" s="73" t="n">
-        <ns0:v>725000</ns0:v>
+        <ns0:v>785000</ns0:v>
       </ns0:c>
       <ns0:c r="AD109" s="74" t="inlineStr">
         <ns0:is>
@@ -11982,7 +11982,7 @@
       </ns0:c>
       <ns0:c r="AF109" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Correção moderada para reforçar a progressão da coluna T2 Sul/Oeste entre pisos.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Correção moderada para reforçar a progressão da coluna T2 Sul/Oeste entre pisos.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG109" s="74" t="inlineStr">
@@ -12081,7 +12081,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC110" s="73" t="n">
-        <ns0:v>400000</ns0:v>
+        <ns0:v>420000</ns0:v>
       </ns0:c>
       <ns0:c r="AD110" s="74" t="inlineStr">
         <ns0:is>
@@ -12095,7 +12095,7 @@
       </ns0:c>
       <ns0:c r="AF110" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG110" s="74" t="inlineStr">
@@ -12194,7 +12194,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC111" s="73" t="n">
-        <ns0:v>500000</ns0:v>
+        <ns0:v>535000</ns0:v>
       </ns0:c>
       <ns0:c r="AD111" s="74" t="inlineStr">
         <ns0:is>
@@ -12208,7 +12208,7 @@
       </ns0:c>
       <ns0:c r="AF111" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG111" s="74" t="inlineStr">
@@ -12307,7 +12307,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC112" s="73" t="n">
-        <ns0:v>475000</ns0:v>
+        <ns0:v>510000</ns0:v>
       </ns0:c>
       <ns0:c r="AD112" s="74" t="inlineStr">
         <ns0:is>
@@ -12321,7 +12321,7 @@
       </ns0:c>
       <ns0:c r="AF112" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG112" s="74" t="inlineStr">
@@ -12420,7 +12420,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC113" s="73" t="n">
-        <ns0:v>735000</ns0:v>
+        <ns0:v>795000</ns0:v>
       </ns0:c>
       <ns0:c r="AD113" s="74" t="inlineStr">
         <ns0:is>
@@ -12434,7 +12434,7 @@
       </ns0:c>
       <ns0:c r="AF113" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T2+1 de área ampla; ajuste contido face aos T2 próximos.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T2+1 de área ampla; ajuste contido face aos T2 próximos.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG113" s="74" t="inlineStr">
@@ -12533,7 +12533,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC114" s="73" t="n">
-        <ns0:v>625000</ns0:v>
+        <ns0:v>675000</ns0:v>
       </ns0:c>
       <ns0:c r="AD114" s="74" t="inlineStr">
         <ns0:is>
@@ -12547,7 +12547,7 @@
       </ns0:c>
       <ns0:c r="AF114" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG114" s="74" t="inlineStr">
@@ -12646,7 +12646,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC115" s="73" t="n">
-        <ns0:v>415000</ns0:v>
+        <ns0:v>425000</ns0:v>
       </ns0:c>
       <ns0:c r="AD115" s="74" t="inlineStr">
         <ns0:is>
@@ -12660,7 +12660,7 @@
       </ns0:c>
       <ns0:c r="AF115" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG115" s="74" t="inlineStr">
@@ -12759,7 +12759,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC116" s="73" t="n">
-        <ns0:v>1000000</ns0:v>
+        <ns0:v>1200000</ns0:v>
       </ns0:c>
       <ns0:c r="AD116" s="74" t="inlineStr">
         <ns0:is>
@@ -12773,7 +12773,7 @@
       </ns0:c>
       <ns0:c r="AF116" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T3 Sul/Este de grande área e exterior relevante; posicionamento abaixo do Apt. 16 preservado.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T3 Sul/Este de grande área e exterior relevante; posicionamento abaixo do Apt. 16 preservado.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG116" s="74" t="inlineStr">
@@ -12872,7 +12872,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC117" s="73" t="n">
-        <ns0:v>775000</ns0:v>
+        <ns0:v>830000</ns0:v>
       </ns0:c>
       <ns0:c r="AD117" s="74" t="inlineStr">
         <ns0:is>
@@ -12886,7 +12886,7 @@
       </ns0:c>
       <ns0:c r="AF117" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Progressão moderada da coluna T2 Sul/Oeste face ao Apt. 2.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Progressão moderada da coluna T2 Sul/Oeste face ao Apt. 2.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG117" s="74" t="inlineStr">
@@ -12985,7 +12985,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC118" s="73" t="n">
-        <ns0:v>415000</ns0:v>
+        <ns0:v>440000</ns0:v>
       </ns0:c>
       <ns0:c r="AD118" s="74" t="inlineStr">
         <ns0:is>
@@ -12999,7 +12999,7 @@
       </ns0:c>
       <ns0:c r="AF118" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG118" s="74" t="inlineStr">
@@ -13098,7 +13098,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC119" s="73" t="n">
-        <ns0:v>465000</ns0:v>
+        <ns0:v>515000</ns0:v>
       </ns0:c>
       <ns0:c r="AD119" s="74" t="inlineStr">
         <ns0:is>
@@ -13112,7 +13112,7 @@
       </ns0:c>
       <ns0:c r="AF119" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG119" s="74" t="inlineStr">
@@ -13211,7 +13211,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC120" s="73" t="n">
-        <ns0:v>465000</ns0:v>
+        <ns0:v>500000</ns0:v>
       </ns0:c>
       <ns0:c r="AD120" s="74" t="inlineStr">
         <ns0:is>
@@ -13225,7 +13225,7 @@
       </ns0:c>
       <ns0:c r="AF120" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Recomendação condicionada à validação das áreas/características da fração face ao Apt. 12.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Recomendação condicionada à validação das áreas/características da fração face ao Apt. 12.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG120" s="74" t="inlineStr">
@@ -13324,7 +13324,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC121" s="73" t="n">
-        <ns0:v>685000</ns0:v>
+        <ns0:v>735000</ns0:v>
       </ns0:c>
       <ns0:c r="AD121" s="74" t="inlineStr">
         <ns0:is>
@@ -13338,7 +13338,7 @@
       </ns0:c>
       <ns0:c r="AF121" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG121" s="74" t="inlineStr">
@@ -13437,7 +13437,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC122" s="73" t="n">
-        <ns0:v>650000</ns0:v>
+        <ns0:v>705000</ns0:v>
       </ns0:c>
       <ns0:c r="AD122" s="74" t="inlineStr">
         <ns0:is>
@@ -13451,7 +13451,7 @@
       </ns0:c>
       <ns0:c r="AF122" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG122" s="74" t="inlineStr">
@@ -13550,7 +13550,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC123" s="73" t="n">
-        <ns0:v>1100000</ns0:v>
+        <ns0:v>1300000</ns0:v>
       </ns0:c>
       <ns0:c r="AD123" s="74" t="inlineStr">
         <ns0:is>
@@ -13564,7 +13564,7 @@
       </ns0:c>
       <ns0:c r="AF123" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG123" s="74" t="inlineStr">
@@ -13663,7 +13663,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC124" s="73" t="n">
-        <ns0:v>825000</ns0:v>
+        <ns0:v>880000</ns0:v>
       </ns0:c>
       <ns0:c r="AD124" s="74" t="inlineStr">
         <ns0:is>
@@ -13677,7 +13677,7 @@
       </ns0:c>
       <ns0:c r="AF124" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Reforço da progressão interna da coluna T2 Sul/Oeste entre os pisos 2, 3 e 4.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Reforço da progressão interna da coluna T2 Sul/Oeste entre os pisos 2, 3 e 4.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG124" s="74" t="inlineStr">
@@ -13776,7 +13776,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC125" s="73" t="n">
-        <ns0:v>450000</ns0:v>
+        <ns0:v>465000</ns0:v>
       </ns0:c>
       <ns0:c r="AD125" s="74" t="inlineStr">
         <ns0:is>
@@ -13790,7 +13790,7 @@
       </ns0:c>
       <ns0:c r="AF125" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG125" s="74" t="inlineStr">
@@ -13889,7 +13889,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC126" s="73" t="n">
-        <ns0:v>385000</ns0:v>
+        <ns0:v>395000</ns0:v>
       </ns0:c>
       <ns0:c r="AD126" s="74" t="inlineStr">
         <ns0:is>
@@ -13903,7 +13903,7 @@
       </ns0:c>
       <ns0:c r="AF126" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG126" s="74" t="inlineStr">
@@ -14002,7 +14002,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC127" s="73" t="n">
-        <ns0:v>435000</ns0:v>
+        <ns0:v>440000</ns0:v>
       </ns0:c>
       <ns0:c r="AD127" s="74" t="inlineStr">
         <ns0:is>
@@ -14016,7 +14016,7 @@
       </ns0:c>
       <ns0:c r="AF127" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG127" s="74" t="inlineStr">
@@ -14115,7 +14115,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC128" s="73" t="n">
-        <ns0:v>675000</ns0:v>
+        <ns0:v>745000</ns0:v>
       </ns0:c>
       <ns0:c r="AD128" s="74" t="inlineStr">
         <ns0:is>
@@ -14129,7 +14129,7 @@
       </ns0:c>
       <ns0:c r="AF128" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T2 Este/Oeste no piso 3; ajuste moderado face aos Apt. 14 e 26.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T2 Este/Oeste no piso 3; ajuste moderado face aos Apt. 14 e 26.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG128" s="74" t="inlineStr">
@@ -14228,7 +14228,7 @@
         <ns0:f t="shared" si="26"/>
       </ns0:c>
       <ns0:c r="AC129" s="73" t="n">
-        <ns0:v>695000</ns0:v>
+        <ns0:v>775000</ns0:v>
       </ns0:c>
       <ns0:c r="AD129" s="74" t="inlineStr">
         <ns0:is>
@@ -14242,7 +14242,7 @@
       </ns0:c>
       <ns0:c r="AF129" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG129" s="74" t="inlineStr">
@@ -14341,7 +14341,7 @@
         <ns0:f t="shared" ref="AB130:AB161" si="32">IF(A130="The View","",IF(OR(J130&lt;2026,Y130="Baixa"),"Alta",IF(W130&lt;0.55,"Média","Baixa")))</ns0:f>
       </ns0:c>
       <ns0:c r="AC130" s="73" t="n">
-        <ns0:v>1000000</ns0:v>
+        <ns0:v>1075000</ns0:v>
       </ns0:c>
       <ns0:c r="AD130" s="74" t="inlineStr">
         <ns0:is>
@@ -14355,7 +14355,7 @@
       </ns0:c>
       <ns0:c r="AF130" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG130" s="74" t="inlineStr">
@@ -14454,7 +14454,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC131" s="73" t="n">
-        <ns0:v>900000</ns0:v>
+        <ns0:v>940000</ns0:v>
       </ns0:c>
       <ns0:c r="AD131" s="74" t="inlineStr">
         <ns0:is>
@@ -14468,7 +14468,7 @@
       </ns0:c>
       <ns0:c r="AF131" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Piso 4, orientação Sul/Oeste e posição premium; reduz diferença excessiva face ao Apt. 23 mantendo Sul/Este valorizado.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Piso 4, orientação Sul/Oeste e posição premium; reduz diferença excessiva face ao Apt. 23 mantendo Sul/Este valorizado.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG131" s="74" t="inlineStr">
@@ -14567,7 +14567,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC132" s="73" t="n">
-        <ns0:v>475000</ns0:v>
+        <ns0:v>490000</ns0:v>
       </ns0:c>
       <ns0:c r="AD132" s="74" t="inlineStr">
         <ns0:is>
@@ -14581,7 +14581,7 @@
       </ns0:c>
       <ns0:c r="AF132" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG132" s="74" t="inlineStr">
@@ -14680,7 +14680,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC133" s="73" t="n">
-        <ns0:v>725000</ns0:v>
+        <ns0:v>815000</ns0:v>
       </ns0:c>
       <ns0:c r="AD133" s="74" t="inlineStr">
         <ns0:is>
@@ -14694,7 +14694,7 @@
       </ns0:c>
       <ns0:c r="AF133" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG133" s="74" t="inlineStr">
@@ -14793,7 +14793,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC134" s="73" t="n">
-        <ns0:v>475000</ns0:v>
+        <ns0:v>510000</ns0:v>
       </ns0:c>
       <ns0:c r="AD134" s="74" t="inlineStr">
         <ns0:is>
@@ -14807,7 +14807,7 @@
       </ns0:c>
       <ns0:c r="AF134" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG134" s="74" t="inlineStr">
@@ -14906,7 +14906,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC135" s="73" t="n">
-        <ns0:v>525000</ns0:v>
+        <ns0:v>565000</ns0:v>
       </ns0:c>
       <ns0:c r="AD135" s="74" t="inlineStr">
         <ns0:is>
@@ -14920,7 +14920,7 @@
       </ns0:c>
       <ns0:c r="AF135" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG135" s="74" t="inlineStr">
@@ -15019,7 +15019,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC136" s="73" t="n">
-        <ns0:v>525000</ns0:v>
+        <ns0:v>545000</ns0:v>
       </ns0:c>
       <ns0:c r="AD136" s="74" t="inlineStr">
         <ns0:is>
@@ -15033,7 +15033,7 @@
       </ns0:c>
       <ns0:c r="AF136" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG136" s="74" t="inlineStr">
@@ -15132,7 +15132,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC137" s="73" t="n">
-        <ns0:v>1100000</ns0:v>
+        <ns0:v>1175000</ns0:v>
       </ns0:c>
       <ns0:c r="AD137" s="74" t="inlineStr">
         <ns0:is>
@@ -15146,7 +15146,7 @@
       </ns0:c>
       <ns0:c r="AF137" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T2 Sul/Este do piso 5; referência técnica premium fora de comercialização.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T2 Sul/Este do piso 5; referência técnica premium fora de comercialização.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG137" s="74" t="inlineStr">
@@ -15264,7 +15264,7 @@
       </ns0:c>
       <ns0:c r="AF138" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço técnico de referência. Fração atualmente fora de comercialização.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço técnico de referência. Fração atualmente fora de comercialização.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG138" s="74" t="inlineStr">
@@ -15368,7 +15368,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC139" s="73" t="n">
-        <ns0:v>500000</ns0:v>
+        <ns0:v>515000</ns0:v>
       </ns0:c>
       <ns0:c r="AD139" s="74" t="inlineStr">
         <ns0:is>
@@ -15382,7 +15382,7 @@
       </ns0:c>
       <ns0:c r="AF139" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T1 do piso 5; referência técnica fora de comercialização.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T1 do piso 5; referência técnica fora de comercialização.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG139" s="74" t="inlineStr">
@@ -15486,7 +15486,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC140" s="73" t="n">
-        <ns0:v>750000</ns0:v>
+        <ns0:v>795000</ns0:v>
       </ns0:c>
       <ns0:c r="AD140" s="74" t="inlineStr">
         <ns0:is>
@@ -15500,7 +15500,7 @@
       </ns0:c>
       <ns0:c r="AF140" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T2 Este/Oeste do piso 5; preço técnico para leitura da coluna, fora de comercialização.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T2 Este/Oeste do piso 5; preço técnico para leitura da coluna, fora de comercialização.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG140" s="74" t="inlineStr">
@@ -15604,7 +15604,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC141" s="73" t="n">
-        <ns0:v>880000</ns0:v>
+        <ns0:v>935000</ns0:v>
       </ns0:c>
       <ns0:c r="AD141" s="74" t="inlineStr">
         <ns0:is>
@@ -15618,7 +15618,7 @@
       </ns0:c>
       <ns0:c r="AF141" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T2 de área ampla no piso 5; referência técnica fora de comercialização.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T2 de área ampla no piso 5; referência técnica fora de comercialização.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG141" s="74" t="inlineStr">
@@ -15722,7 +15722,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC142" s="73" t="n">
-        <ns0:v>700000</ns0:v>
+        <ns0:v>800000</ns0:v>
       </ns0:c>
       <ns0:c r="AD142" s="74" t="inlineStr">
         <ns0:is>
@@ -15736,7 +15736,7 @@
       </ns0:c>
       <ns0:c r="AF142" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Duplex singular no piso 5; referência técnica fora de comercialização.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Duplex singular no piso 5; referência técnica fora de comercialização.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG142" s="74" t="inlineStr">
@@ -15840,7 +15840,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC143" s="73" t="n">
-        <ns0:v>1500000</ns0:v>
+        <ns0:v>1750000</ns0:v>
       </ns0:c>
       <ns0:c r="AD143" s="74" t="inlineStr">
         <ns0:is>
@@ -15854,7 +15854,7 @@
       </ns0:c>
       <ns0:c r="AF143" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço elevado mas suportado pelo posicionamento premium, piso 6, orientação Sul/Este e benchmark waterfront.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço elevado mas suportado pelo posicionamento premium, piso 6, orientação Sul/Este e benchmark waterfront.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG143" s="74" t="inlineStr">
@@ -15953,7 +15953,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC144" s="73" t="n">
-        <ns0:v>1105000</ns0:v>
+        <ns0:v>1150000</ns0:v>
       </ns0:c>
       <ns0:c r="AD144" s="74" t="inlineStr">
         <ns0:is>
@@ -15967,7 +15967,7 @@
       </ns0:c>
       <ns0:c r="AF144" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG144" s="74" t="inlineStr">
@@ -16066,7 +16066,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC145" s="73" t="n">
-        <ns0:v>490000</ns0:v>
+        <ns0:v>545000</ns0:v>
       </ns0:c>
       <ns0:c r="AD145" s="74" t="inlineStr">
         <ns0:is>
@@ -16080,7 +16080,7 @@
       </ns0:c>
       <ns0:c r="AF145" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): Preço base tecnicamente alinhado com a concorrência interna e o posicionamento da fração.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG145" s="74" t="inlineStr">
@@ -16179,7 +16179,7 @@
         <ns0:f t="shared" si="32"/>
       </ns0:c>
       <ns0:c r="AC146" s="73" t="n">
-        <ns0:v>1150000</ns0:v>
+        <ns0:v>1300000</ns0:v>
       </ns0:c>
       <ns0:c r="AD146" s="74" t="inlineStr">
         <ns0:is>
@@ -16193,7 +16193,7 @@
       </ns0:c>
       <ns0:c r="AF146" s="74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Preço recomendado definido pela gestão em outubro de 2026. Não resulta de cálculo automático do compset. Enquadramento anterior (setembro de 2026): T3 no último piso com exterior excecional; mantém prémio sobre o T2 Apt. 37 apesar da orientação inferior.</ns0:t>
+          <ns0:t>Preço recomendado da análise independente de outubro de 2026, conforme tabela técnica validada. Não substitui o preço comercial atual. Enquadramento anterior (setembro de 2026): T3 no último piso com exterior excecional; mantém prémio sobre o T2 Apt. 37 apesar da orientação inferior.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="AG146" s="74" t="inlineStr">
@@ -62522,11 +62522,11 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B24" s="95" t="n">
-        <ns0:v>27395000</ns0:v>
+        <ns0:v>29675000</ns0:v>
       </ns0:c>
       <ns0:c r="C24" s="94" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gestão · outubro 2026; não altera PVP ou valores comerciais.</ns0:t>
+          <ns0:t>Análise independente · outubro 2026; não altera PVP ou preços comerciais atuais.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D24" s="94"/>

</xml_diff>